<commit_message>
Update 25-04 VBI data and fix VBI_TT08 import columns
</commit_message>
<xml_diff>
--- a/f_total.xlsx
+++ b/f_total.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\Downloads\GBOC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\GBOC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92273AB-3FF6-4EB3-BA46-F28314A9921F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574D097D-A6FF-4456-88AB-069364007947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45E122DF-0947-42F2-896B-598FAC0AE8C4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{45E122DF-0947-42F2-896B-598FAC0AE8C4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="47">
   <si>
     <t>AGG</t>
   </si>
@@ -168,6 +168,18 @@
   </si>
   <si>
     <t>KH giao</t>
+  </si>
+  <si>
+    <t>Đầu kỳ CMT</t>
+  </si>
+  <si>
+    <t>Đầu kỳ yếu thế</t>
+  </si>
+  <si>
+    <t>Đầu kỳ còn lại</t>
+  </si>
+  <si>
+    <t>TH ngày 18</t>
   </si>
 </sst>
 </file>
@@ -238,7 +250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -253,13 +265,17 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -597,17 +613,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F8CCBB-734C-484D-BA4E-0EDC445F6339}">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.625" customWidth="1"/>
-    <col min="5" max="5" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.125" customWidth="1"/>
-    <col min="8" max="8" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="12.625" customWidth="1"/>
+    <col min="7" max="7" width="12.625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="12.625" customWidth="1"/>
+    <col min="9" max="9" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -618,19 +635,31 @@
         <v>37</v>
       </c>
       <c r="D1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
         <v>42</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -640,23 +669,28 @@
       <c r="C2" s="4">
         <v>1079493</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6">
+        <v>298044</v>
+      </c>
+      <c r="G2" s="9">
+        <v>33269</v>
+      </c>
+      <c r="H2" s="6">
         <v>231171</v>
       </c>
-      <c r="E2" s="1">
+      <c r="I2" s="1">
         <v>13679</v>
       </c>
-      <c r="F2" s="1">
+      <c r="J2" s="1">
         <v>80702</v>
       </c>
-      <c r="G2" s="1">
+      <c r="K2" s="1">
         <v>150469</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -666,23 +700,28 @@
       <c r="C3" s="4">
         <v>1285128</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6">
+        <v>419726</v>
+      </c>
+      <c r="G3" s="9">
+        <v>86085</v>
+      </c>
+      <c r="H3" s="6">
         <v>275954</v>
       </c>
-      <c r="E3" s="1">
+      <c r="I3" s="1">
         <v>7402.545454545455</v>
       </c>
-      <c r="F3" s="1">
+      <c r="J3" s="1">
         <v>194526</v>
       </c>
-      <c r="G3" s="1">
+      <c r="K3" s="1">
         <v>81428</v>
       </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -692,23 +731,28 @@
       <c r="C4" s="4">
         <v>183942</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6">
+        <v>30112</v>
+      </c>
+      <c r="G4" s="9">
+        <v>14085</v>
+      </c>
+      <c r="H4" s="6">
         <v>39843</v>
       </c>
-      <c r="E4" s="1">
+      <c r="I4" s="1">
         <v>1701.1818181818182</v>
       </c>
-      <c r="F4" s="1">
+      <c r="J4" s="1">
         <v>21130</v>
       </c>
-      <c r="G4" s="1">
+      <c r="K4" s="1">
         <v>18713</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -718,23 +762,28 @@
       <c r="C5" s="4">
         <v>294606</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6">
+        <v>76246</v>
+      </c>
+      <c r="G5" s="9">
+        <v>9460</v>
+      </c>
+      <c r="H5" s="6">
         <v>64997</v>
       </c>
-      <c r="E5" s="1">
+      <c r="I5" s="1">
         <v>3855.2727272727275</v>
       </c>
-      <c r="F5" s="1">
+      <c r="J5" s="1">
         <v>22589</v>
       </c>
-      <c r="G5" s="1">
+      <c r="K5" s="1">
         <v>42408</v>
       </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -744,23 +793,28 @@
       <c r="C6" s="4">
         <v>853784</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6">
+        <v>257665</v>
+      </c>
+      <c r="G6" s="9">
+        <v>26774</v>
+      </c>
+      <c r="H6" s="6">
         <v>183356</v>
       </c>
-      <c r="E6" s="1">
+      <c r="I6" s="1">
         <v>10676.272727272728</v>
       </c>
-      <c r="F6" s="1">
+      <c r="J6" s="1">
         <v>65917</v>
       </c>
-      <c r="G6" s="1">
+      <c r="K6" s="1">
         <v>117439</v>
       </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -770,23 +824,28 @@
       <c r="C7" s="4">
         <v>145885</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6">
+        <v>42222</v>
+      </c>
+      <c r="G7" s="9">
+        <v>6199</v>
+      </c>
+      <c r="H7" s="6">
         <v>32296</v>
       </c>
-      <c r="E7" s="1">
+      <c r="I7" s="1">
         <v>1734.1818181818182</v>
       </c>
-      <c r="F7" s="1">
+      <c r="J7" s="1">
         <v>13220</v>
       </c>
-      <c r="G7" s="1">
+      <c r="K7" s="1">
         <v>19076</v>
       </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -796,23 +855,28 @@
       <c r="C8" s="4">
         <v>865857</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6">
+        <v>187915</v>
+      </c>
+      <c r="G8" s="9">
+        <v>60289</v>
+      </c>
+      <c r="H8" s="6">
         <v>185241</v>
       </c>
-      <c r="E8" s="1">
+      <c r="I8" s="1">
         <v>7546.727272727273</v>
       </c>
-      <c r="F8" s="1">
+      <c r="J8" s="1">
         <v>102227</v>
       </c>
-      <c r="G8" s="1">
+      <c r="K8" s="1">
         <v>83014</v>
       </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -822,23 +886,28 @@
       <c r="C9" s="4">
         <v>645765</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6">
+        <v>172446</v>
+      </c>
+      <c r="G9" s="9">
+        <v>36956</v>
+      </c>
+      <c r="H9" s="6">
         <v>138279</v>
       </c>
-      <c r="E9" s="1">
+      <c r="I9" s="1">
         <v>5918.818181818182</v>
       </c>
-      <c r="F9" s="1">
+      <c r="J9" s="1">
         <v>73172</v>
       </c>
-      <c r="G9" s="1">
+      <c r="K9" s="1">
         <v>65107</v>
       </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -848,23 +917,28 @@
       <c r="C10" s="4">
         <v>1409894</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6">
+        <v>425517</v>
+      </c>
+      <c r="G10" s="9">
+        <v>75045</v>
+      </c>
+      <c r="H10" s="6">
         <v>301559</v>
       </c>
-      <c r="E10" s="1">
+      <c r="I10" s="1">
         <v>13768.272727272728</v>
       </c>
-      <c r="F10" s="1">
+      <c r="J10" s="1">
         <v>150108</v>
       </c>
-      <c r="G10" s="1">
+      <c r="K10" s="1">
         <v>151451</v>
       </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -874,23 +948,28 @@
       <c r="C11" s="4">
         <v>1007603</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6">
+        <v>274111</v>
+      </c>
+      <c r="G11" s="9">
+        <v>43552</v>
+      </c>
+      <c r="H11" s="6">
         <v>214388</v>
       </c>
-      <c r="E11" s="1">
+      <c r="I11" s="1">
         <v>11592.454545454546</v>
       </c>
-      <c r="F11" s="1">
+      <c r="J11" s="1">
         <v>86871</v>
       </c>
-      <c r="G11" s="1">
+      <c r="K11" s="1">
         <v>127517</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -900,23 +979,28 @@
       <c r="C12" s="4">
         <v>1084925</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6">
+        <v>258292</v>
+      </c>
+      <c r="G12" s="9">
+        <v>61332</v>
+      </c>
+      <c r="H12" s="6">
         <v>232427</v>
       </c>
-      <c r="E12" s="1">
+      <c r="I12" s="1">
         <v>11115.09090909091</v>
       </c>
-      <c r="F12" s="1">
+      <c r="J12" s="1">
         <v>110161</v>
       </c>
-      <c r="G12" s="1">
+      <c r="K12" s="1">
         <v>122266</v>
       </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -926,23 +1010,28 @@
       <c r="C13" s="4">
         <v>3578511</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6">
+        <v>1393293</v>
+      </c>
+      <c r="G13" s="9">
+        <v>135141</v>
+      </c>
+      <c r="H13" s="6">
         <v>766690</v>
       </c>
-      <c r="E13" s="1">
+      <c r="I13" s="1">
         <v>36311.36363636364</v>
       </c>
-      <c r="F13" s="1">
+      <c r="J13" s="1">
         <v>367265</v>
       </c>
-      <c r="G13" s="1">
+      <c r="K13" s="1">
         <v>399425</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -952,23 +1041,28 @@
       <c r="C14" s="4">
         <v>3265949</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6">
+        <v>1559361</v>
+      </c>
+      <c r="G14" s="9">
+        <v>122051</v>
+      </c>
+      <c r="H14" s="6">
         <v>699078</v>
       </c>
-      <c r="E14" s="1">
+      <c r="I14" s="1">
         <v>24981.363636363636</v>
       </c>
-      <c r="F14" s="1">
+      <c r="J14" s="1">
         <v>424283</v>
       </c>
-      <c r="G14" s="1">
+      <c r="K14" s="1">
         <v>274795</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -978,23 +1072,28 @@
       <c r="C15" s="4">
         <v>1044956</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6">
+        <v>424815</v>
+      </c>
+      <c r="G15" s="9">
+        <v>49488</v>
+      </c>
+      <c r="H15" s="6">
         <v>224183</v>
       </c>
-      <c r="E15" s="1">
+      <c r="I15" s="1">
         <v>7320.909090909091</v>
       </c>
-      <c r="F15" s="1">
+      <c r="J15" s="1">
         <v>143653</v>
       </c>
-      <c r="G15" s="1">
+      <c r="K15" s="1">
         <v>80530</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-    </row>
-    <row r="16" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
@@ -1004,23 +1103,28 @@
       <c r="C16" s="5">
         <v>361645</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7">
+        <v>87356</v>
+      </c>
+      <c r="G16" s="9">
+        <v>28585</v>
+      </c>
+      <c r="H16" s="7">
         <v>77637</v>
       </c>
-      <c r="E16" s="1">
+      <c r="I16" s="1">
         <v>1452.2727272727273</v>
       </c>
-      <c r="F16" s="1">
+      <c r="J16" s="1">
         <v>61662</v>
       </c>
-      <c r="G16" s="1">
+      <c r="K16" s="1">
         <v>15975</v>
       </c>
-      <c r="H16" s="1"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -1030,23 +1134,28 @@
       <c r="C17" s="4">
         <v>285109</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6">
+        <v>75597</v>
+      </c>
+      <c r="G17" s="9">
+        <v>18705</v>
+      </c>
+      <c r="H17" s="6">
         <v>61076</v>
       </c>
-      <c r="E17" s="1">
+      <c r="I17" s="1">
         <v>2414.909090909091</v>
       </c>
-      <c r="F17" s="1">
+      <c r="J17" s="1">
         <v>34512</v>
       </c>
-      <c r="G17" s="1">
+      <c r="K17" s="1">
         <v>26564</v>
       </c>
-      <c r="H17" s="1"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -1056,23 +1165,28 @@
       <c r="C18" s="4">
         <v>894371</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6">
+        <v>338319</v>
+      </c>
+      <c r="G18" s="9">
+        <v>52801</v>
+      </c>
+      <c r="H18" s="6">
         <v>190950</v>
       </c>
-      <c r="E18" s="1">
+      <c r="I18" s="1">
         <v>6069.454545454545</v>
       </c>
-      <c r="F18" s="1">
+      <c r="J18" s="1">
         <v>124186</v>
       </c>
-      <c r="G18" s="1">
+      <c r="K18" s="1">
         <v>66764</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -1082,23 +1196,28 @@
       <c r="C19" s="4">
         <v>565397</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6">
+        <v>129712</v>
+      </c>
+      <c r="G19" s="9">
+        <v>36512</v>
+      </c>
+      <c r="H19" s="6">
         <v>120456</v>
       </c>
-      <c r="E19" s="1">
+      <c r="I19" s="1">
         <v>5021</v>
       </c>
-      <c r="F19" s="1">
+      <c r="J19" s="1">
         <v>65225</v>
       </c>
-      <c r="G19" s="1">
+      <c r="K19" s="1">
         <v>55231</v>
       </c>
-      <c r="H19" s="1"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -1108,23 +1227,28 @@
       <c r="C20" s="4">
         <v>526562</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6">
+        <v>127241</v>
+      </c>
+      <c r="G20" s="9">
+        <v>28925</v>
+      </c>
+      <c r="H20" s="6">
         <v>113964</v>
       </c>
-      <c r="E20" s="1">
+      <c r="I20" s="1">
         <v>5339.727272727273</v>
       </c>
-      <c r="F20" s="1">
+      <c r="J20" s="1">
         <v>55227</v>
       </c>
-      <c r="G20" s="1">
+      <c r="K20" s="1">
         <v>58737</v>
       </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -1134,23 +1258,28 @@
       <c r="C21" s="4">
         <v>162492</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6">
+        <v>36211</v>
+      </c>
+      <c r="G21" s="9">
+        <v>4271</v>
+      </c>
+      <c r="H21" s="6">
         <v>35928</v>
       </c>
-      <c r="E21" s="1">
+      <c r="I21" s="1">
         <v>2216.5454545454545</v>
       </c>
-      <c r="F21" s="1">
+      <c r="J21" s="1">
         <v>11546</v>
       </c>
-      <c r="G21" s="1">
+      <c r="K21" s="1">
         <v>24382</v>
       </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -1160,23 +1289,28 @@
       <c r="C22" s="4">
         <v>1188375</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6">
+        <v>281213</v>
+      </c>
+      <c r="G22" s="9">
+        <v>49983</v>
+      </c>
+      <c r="H22" s="6">
         <v>254618</v>
       </c>
-      <c r="E22" s="1">
+      <c r="I22" s="1">
         <v>13839</v>
       </c>
-      <c r="F22" s="1">
+      <c r="J22" s="1">
         <v>102389</v>
       </c>
-      <c r="G22" s="1">
+      <c r="K22" s="1">
         <v>152229</v>
       </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -1186,23 +1320,28 @@
       <c r="C23" s="4">
         <v>371038</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6">
+        <v>88344</v>
+      </c>
+      <c r="G23" s="9">
+        <v>20848</v>
+      </c>
+      <c r="H23" s="6">
         <v>79486</v>
       </c>
-      <c r="E23" s="1">
+      <c r="I23" s="1">
         <v>3715.181818181818</v>
       </c>
-      <c r="F23" s="1">
+      <c r="J23" s="1">
         <v>38619</v>
       </c>
-      <c r="G23" s="1">
+      <c r="K23" s="1">
         <v>40867</v>
       </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -1212,23 +1351,28 @@
       <c r="C24" s="4">
         <v>1017106</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6">
+        <v>245892</v>
+      </c>
+      <c r="G24" s="9">
+        <v>68931</v>
+      </c>
+      <c r="H24" s="6">
         <v>217875</v>
       </c>
-      <c r="E24" s="1">
+      <c r="I24" s="1">
         <v>8072.545454545455</v>
       </c>
-      <c r="F24" s="1">
+      <c r="J24" s="1">
         <v>129077</v>
       </c>
-      <c r="G24" s="1">
+      <c r="K24" s="1">
         <v>88798</v>
       </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -1238,23 +1382,28 @@
       <c r="C25" s="4">
         <v>914401</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6">
+        <v>341001</v>
+      </c>
+      <c r="G25" s="9">
+        <v>49929</v>
+      </c>
+      <c r="H25" s="6">
         <v>195226</v>
       </c>
-      <c r="E25" s="1">
+      <c r="I25" s="1">
         <v>7872.727272727273</v>
       </c>
-      <c r="F25" s="1">
+      <c r="J25" s="1">
         <v>108626</v>
       </c>
-      <c r="G25" s="1">
+      <c r="K25" s="1">
         <v>86600</v>
       </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -1264,23 +1413,28 @@
       <c r="C26" s="4">
         <v>1261095</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6">
+        <v>387874</v>
+      </c>
+      <c r="G26" s="9">
+        <v>83582</v>
+      </c>
+      <c r="H26" s="6">
         <v>269506</v>
       </c>
-      <c r="E26" s="1">
+      <c r="I26" s="1">
         <v>8691.363636363636</v>
       </c>
-      <c r="F26" s="1">
+      <c r="J26" s="1">
         <v>173901</v>
       </c>
-      <c r="G26" s="1">
+      <c r="K26" s="1">
         <v>95605</v>
       </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -1290,23 +1444,28 @@
       <c r="C27" s="4">
         <v>416872</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6">
+        <v>160366</v>
+      </c>
+      <c r="G27" s="9">
+        <v>19902</v>
+      </c>
+      <c r="H27" s="6">
         <v>89232</v>
       </c>
-      <c r="E27" s="1">
+      <c r="I27" s="1">
         <v>3199.7272727272725</v>
       </c>
-      <c r="F27" s="1">
+      <c r="J27" s="1">
         <v>54035</v>
       </c>
-      <c r="G27" s="1">
+      <c r="K27" s="1">
         <v>35197</v>
       </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -1316,23 +1475,28 @@
       <c r="C28" s="4">
         <v>576110</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6">
+        <v>130368</v>
+      </c>
+      <c r="G28" s="9">
+        <v>42884</v>
+      </c>
+      <c r="H28" s="6">
         <v>123576</v>
       </c>
-      <c r="E28" s="1">
+      <c r="I28" s="1">
         <v>4800</v>
       </c>
-      <c r="F28" s="1">
+      <c r="J28" s="1">
         <v>70776</v>
       </c>
-      <c r="G28" s="1">
+      <c r="K28" s="1">
         <v>52800</v>
       </c>
-      <c r="H28" s="1"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -1342,23 +1506,28 @@
       <c r="C29" s="4">
         <v>322028</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6">
+        <v>86131</v>
+      </c>
+      <c r="G29" s="9">
+        <v>17942</v>
+      </c>
+      <c r="H29" s="6">
         <v>69184</v>
       </c>
-      <c r="E29" s="1">
+      <c r="I29" s="1">
         <v>3099.3636363636365</v>
       </c>
-      <c r="F29" s="1">
+      <c r="J29" s="1">
         <v>35091</v>
       </c>
-      <c r="G29" s="1">
+      <c r="K29" s="1">
         <v>34093</v>
       </c>
-      <c r="H29" s="1"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -1368,23 +1537,28 @@
       <c r="C30" s="4">
         <v>472333</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6">
+        <v>112163</v>
+      </c>
+      <c r="G30" s="9">
+        <v>20557</v>
+      </c>
+      <c r="H30" s="6">
         <v>102301</v>
       </c>
-      <c r="E30" s="1">
+      <c r="I30" s="1">
         <v>5410.818181818182</v>
       </c>
-      <c r="F30" s="1">
+      <c r="J30" s="1">
         <v>42782</v>
       </c>
-      <c r="G30" s="1">
+      <c r="K30" s="1">
         <v>59519</v>
       </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -1394,23 +1568,28 @@
       <c r="C31" s="4">
         <v>978536</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6">
+        <v>312801</v>
+      </c>
+      <c r="G31" s="9">
+        <v>45959</v>
+      </c>
+      <c r="H31" s="6">
         <v>209020</v>
       </c>
-      <c r="E31" s="1">
+      <c r="I31" s="1">
         <v>10110.454545454546</v>
       </c>
-      <c r="F31" s="1">
+      <c r="J31" s="1">
         <v>97805</v>
       </c>
-      <c r="G31" s="1">
+      <c r="K31" s="1">
         <v>111215</v>
       </c>
-      <c r="H31" s="1"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -1420,23 +1599,28 @@
       <c r="C32" s="4">
         <v>1009008</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6">
+        <v>342337</v>
+      </c>
+      <c r="G32" s="9">
+        <v>33008</v>
+      </c>
+      <c r="H32" s="6">
         <v>215467</v>
       </c>
-      <c r="E32" s="1">
+      <c r="I32" s="1">
         <v>12329.09090909091</v>
       </c>
-      <c r="F32" s="1">
+      <c r="J32" s="1">
         <v>79847</v>
       </c>
-      <c r="G32" s="1">
+      <c r="K32" s="1">
         <v>135620</v>
       </c>
-      <c r="H32" s="1"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -1446,23 +1630,28 @@
       <c r="C33" s="4">
         <v>598334</v>
       </c>
-      <c r="D33" s="7">
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6">
+        <v>170531</v>
+      </c>
+      <c r="G33" s="9">
+        <v>42826</v>
+      </c>
+      <c r="H33" s="6">
         <v>128017</v>
       </c>
-      <c r="E33" s="1">
+      <c r="I33" s="1">
         <v>4191.636363636364</v>
       </c>
-      <c r="F33" s="1">
+      <c r="J33" s="1">
         <v>81909</v>
       </c>
-      <c r="G33" s="1">
+      <c r="K33" s="1">
         <v>46108</v>
       </c>
-      <c r="H33" s="1"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -1472,23 +1661,28 @@
       <c r="C34" s="4">
         <v>619422</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6">
+        <v>150535</v>
+      </c>
+      <c r="G34" s="9">
+        <v>30397</v>
+      </c>
+      <c r="H34" s="6">
         <v>133210</v>
       </c>
-      <c r="E34" s="1">
+      <c r="I34" s="1">
         <v>6730.454545454545</v>
       </c>
-      <c r="F34" s="1">
+      <c r="J34" s="1">
         <v>59175</v>
       </c>
-      <c r="G34" s="1">
+      <c r="K34" s="1">
         <v>74035</v>
       </c>
-      <c r="H34" s="1"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -1498,23 +1692,28 @@
       <c r="C35" s="4">
         <v>1040674</v>
       </c>
-      <c r="D35" s="7">
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6">
+        <v>292375</v>
+      </c>
+      <c r="G35" s="9">
+        <v>43472</v>
+      </c>
+      <c r="H35" s="6">
         <v>221968</v>
       </c>
-      <c r="E35" s="1">
+      <c r="I35" s="1">
         <v>12219.181818181818</v>
       </c>
-      <c r="F35" s="1">
+      <c r="J35" s="1">
         <v>87557</v>
       </c>
-      <c r="G35" s="1">
+      <c r="K35" s="1">
         <v>134411</v>
       </c>
-      <c r="H35" s="1"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>0</v>
       </c>
@@ -1524,20 +1723,28 @@
       <c r="C36" s="1">
         <v>777063</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="10">
+        <v>463874</v>
+      </c>
+      <c r="E36" s="1">
+        <v>313189</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1">
         <v>127144</v>
       </c>
-      <c r="E36" s="1">
+      <c r="I36" s="1">
         <v>8534.0909090909099</v>
       </c>
-      <c r="F36" s="1">
+      <c r="J36" s="1">
         <v>33269</v>
       </c>
-      <c r="G36" s="1">
+      <c r="K36" s="1">
         <v>93875</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>1</v>
       </c>
@@ -1547,20 +1754,28 @@
       <c r="C37" s="1">
         <v>855156</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="10">
+        <v>625314</v>
+      </c>
+      <c r="E37" s="1">
+        <v>229842</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1">
         <v>151775</v>
       </c>
-      <c r="E37" s="1">
+      <c r="I37" s="1">
         <v>5971.818181818182</v>
       </c>
-      <c r="F37" s="1">
+      <c r="J37" s="1">
         <v>86085</v>
       </c>
-      <c r="G37" s="1">
+      <c r="K37" s="1">
         <v>65690</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>2</v>
       </c>
@@ -1570,20 +1785,28 @@
       <c r="C38" s="1">
         <v>153708</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="10">
+        <v>84115</v>
+      </c>
+      <c r="E38" s="1">
+        <v>69593</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1">
         <v>21914</v>
       </c>
-      <c r="E38" s="1">
+      <c r="I38" s="1">
         <v>711.72727272727275</v>
       </c>
-      <c r="F38" s="1">
+      <c r="J38" s="1">
         <v>14085</v>
       </c>
-      <c r="G38" s="1">
+      <c r="K38" s="1">
         <v>7829</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>3</v>
       </c>
@@ -1593,20 +1816,28 @@
       <c r="C39" s="1">
         <v>216463</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="10">
+        <v>101189</v>
+      </c>
+      <c r="E39" s="1">
+        <v>115274</v>
+      </c>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1">
         <v>35749</v>
       </c>
-      <c r="E39" s="1">
+      <c r="I39" s="1">
         <v>2389.909090909091</v>
       </c>
-      <c r="F39" s="1">
+      <c r="J39" s="1">
         <v>9460</v>
       </c>
-      <c r="G39" s="1">
+      <c r="K39" s="1">
         <v>26289</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>4</v>
       </c>
@@ -1616,20 +1847,28 @@
       <c r="C40" s="1">
         <v>590772</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="10">
+        <v>337445</v>
+      </c>
+      <c r="E40" s="1">
+        <v>253327</v>
+      </c>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1">
         <v>100846</v>
       </c>
-      <c r="E40" s="1">
+      <c r="I40" s="1">
         <v>6733.818181818182</v>
       </c>
-      <c r="F40" s="1">
+      <c r="J40" s="1">
         <v>26774</v>
       </c>
-      <c r="G40" s="1">
+      <c r="K40" s="1">
         <v>74072</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>5</v>
       </c>
@@ -1639,20 +1878,28 @@
       <c r="C41" s="1">
         <v>103347</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="10">
+        <v>46238</v>
+      </c>
+      <c r="E41" s="1">
+        <v>57109</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1">
         <v>17763</v>
       </c>
-      <c r="E41" s="1">
+      <c r="I41" s="1">
         <v>1051.2727272727273</v>
       </c>
-      <c r="F41" s="1">
+      <c r="J41" s="1">
         <v>6199</v>
       </c>
-      <c r="G41" s="1">
+      <c r="K41" s="1">
         <v>11564</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1662,20 +1909,28 @@
       <c r="C42" s="1">
         <v>675934</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="10">
+        <v>404500</v>
+      </c>
+      <c r="E42" s="1">
+        <v>271434</v>
+      </c>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1">
         <v>101883</v>
       </c>
-      <c r="E42" s="1">
+      <c r="I42" s="1">
         <v>3781.2727272727275</v>
       </c>
-      <c r="F42" s="1">
+      <c r="J42" s="1">
         <v>60289</v>
       </c>
-      <c r="G42" s="1">
+      <c r="K42" s="1">
         <v>41594</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>7</v>
       </c>
@@ -1685,20 +1940,28 @@
       <c r="C43" s="1">
         <v>470034</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="10">
+        <v>280731</v>
+      </c>
+      <c r="E43" s="1">
+        <v>189303</v>
+      </c>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1">
         <v>76053</v>
       </c>
-      <c r="E43" s="1">
+      <c r="I43" s="1">
         <v>3554.2727272727275</v>
       </c>
-      <c r="F43" s="1">
+      <c r="J43" s="1">
         <v>36956</v>
       </c>
-      <c r="G43" s="1">
+      <c r="K43" s="1">
         <v>39097</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>8</v>
       </c>
@@ -1708,20 +1971,28 @@
       <c r="C44" s="1">
         <v>977311</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="10">
+        <v>656794</v>
+      </c>
+      <c r="E44" s="1">
+        <v>320517</v>
+      </c>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1">
         <v>165858</v>
       </c>
-      <c r="E44" s="1">
+      <c r="I44" s="1">
         <v>8255.7272727272721</v>
       </c>
-      <c r="F44" s="1">
+      <c r="J44" s="1">
         <v>75045</v>
       </c>
-      <c r="G44" s="1">
+      <c r="K44" s="1">
         <v>90813</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>9</v>
       </c>
@@ -1731,20 +2002,28 @@
       <c r="C45" s="1">
         <v>729187</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="10">
+        <v>471388</v>
+      </c>
+      <c r="E45" s="1">
+        <v>257799</v>
+      </c>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1">
         <v>117914</v>
       </c>
-      <c r="E45" s="1">
+      <c r="I45" s="1">
         <v>6760.181818181818</v>
       </c>
-      <c r="F45" s="1">
+      <c r="J45" s="1">
         <v>43552</v>
       </c>
-      <c r="G45" s="1">
+      <c r="K45" s="1">
         <v>74362</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>10</v>
       </c>
@@ -1754,20 +2033,28 @@
       <c r="C46" s="1">
         <v>823905</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="10">
+        <v>494965</v>
+      </c>
+      <c r="E46" s="1">
+        <v>328940</v>
+      </c>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1">
         <v>127835</v>
       </c>
-      <c r="E46" s="1">
+      <c r="I46" s="1">
         <v>6045.727272727273</v>
       </c>
-      <c r="F46" s="1">
+      <c r="J46" s="1">
         <v>61332</v>
       </c>
-      <c r="G46" s="1">
+      <c r="K46" s="1">
         <v>66503</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>11</v>
       </c>
@@ -1777,20 +2064,28 @@
       <c r="C47" s="1">
         <v>2150183</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="10">
+        <v>1412640</v>
+      </c>
+      <c r="E47" s="1">
+        <v>737543</v>
+      </c>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1">
         <v>421680</v>
       </c>
-      <c r="E47" s="1">
+      <c r="I47" s="1">
         <v>26049</v>
       </c>
-      <c r="F47" s="1">
+      <c r="J47" s="1">
         <v>135141</v>
       </c>
-      <c r="G47" s="1">
+      <c r="K47" s="1">
         <v>286539</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>12</v>
       </c>
@@ -1800,20 +2095,28 @@
       <c r="C48" s="1">
         <v>1663325</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="10">
+        <v>1085932</v>
+      </c>
+      <c r="E48" s="1">
+        <v>577393</v>
+      </c>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1">
         <v>384493</v>
       </c>
-      <c r="E48" s="1">
+      <c r="I48" s="1">
         <v>23858.363636363636</v>
       </c>
-      <c r="F48" s="1">
+      <c r="J48" s="1">
         <v>122051</v>
       </c>
-      <c r="G48" s="1">
+      <c r="K48" s="1">
         <v>262442</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>13</v>
       </c>
@@ -1823,20 +2126,28 @@
       <c r="C49" s="1">
         <v>610852</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="10">
+        <v>399689</v>
+      </c>
+      <c r="E49" s="1">
+        <v>211163</v>
+      </c>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1">
         <v>123301</v>
       </c>
-      <c r="E49" s="1">
+      <c r="I49" s="1">
         <v>6710.272727272727</v>
       </c>
-      <c r="F49" s="1">
+      <c r="J49" s="1">
         <v>49488</v>
       </c>
-      <c r="G49" s="1">
+      <c r="K49" s="1">
         <v>73813</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>14</v>
       </c>
@@ -1846,20 +2157,28 @@
       <c r="C50" s="1">
         <v>272950</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="10">
+        <v>182356</v>
+      </c>
+      <c r="E50" s="1">
+        <v>90594</v>
+      </c>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1">
         <v>42700</v>
       </c>
-      <c r="E50" s="1">
+      <c r="I50" s="1">
         <v>1283.1818181818182</v>
       </c>
-      <c r="F50" s="1">
+      <c r="J50" s="1">
         <v>28585</v>
       </c>
-      <c r="G50" s="1">
+      <c r="K50" s="1">
         <v>14115</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>15</v>
       </c>
@@ -1869,20 +2188,28 @@
       <c r="C51" s="1">
         <v>207766</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="10">
+        <v>141794</v>
+      </c>
+      <c r="E51" s="1">
+        <v>65972</v>
+      </c>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1">
         <v>33592</v>
       </c>
-      <c r="E51" s="1">
+      <c r="I51" s="1">
         <v>1353.3636363636363</v>
       </c>
-      <c r="F51" s="1">
+      <c r="J51" s="1">
         <v>18705</v>
       </c>
-      <c r="G51" s="1">
+      <c r="K51" s="1">
         <v>14887</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>16</v>
       </c>
@@ -1892,20 +2219,28 @@
       <c r="C52" s="1">
         <v>549163</v>
       </c>
-      <c r="D52" s="1">
+      <c r="D52" s="10">
+        <v>341243</v>
+      </c>
+      <c r="E52" s="1">
+        <v>207920</v>
+      </c>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1">
         <v>105023</v>
       </c>
-      <c r="E52" s="1">
+      <c r="I52" s="1">
         <v>4747.454545454545</v>
       </c>
-      <c r="F52" s="1">
+      <c r="J52" s="1">
         <v>52801</v>
       </c>
-      <c r="G52" s="1">
+      <c r="K52" s="1">
         <v>52222</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>17</v>
       </c>
@@ -1915,20 +2250,28 @@
       <c r="C53" s="1">
         <v>433574</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="10">
+        <v>294518</v>
+      </c>
+      <c r="E53" s="1">
+        <v>139056</v>
+      </c>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1">
         <v>66251</v>
       </c>
-      <c r="E53" s="1">
+      <c r="I53" s="1">
         <v>2703.5454545454545</v>
       </c>
-      <c r="F53" s="1">
+      <c r="J53" s="1">
         <v>36512</v>
       </c>
-      <c r="G53" s="1">
+      <c r="K53" s="1">
         <v>29739</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>18</v>
       </c>
@@ -1938,20 +2281,28 @@
       <c r="C54" s="1">
         <v>398499</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="10">
+        <v>203892</v>
+      </c>
+      <c r="E54" s="1">
+        <v>194607</v>
+      </c>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1">
         <v>62680</v>
       </c>
-      <c r="E54" s="1">
+      <c r="I54" s="1">
         <v>3068.6363636363635</v>
       </c>
-      <c r="F54" s="1">
+      <c r="J54" s="1">
         <v>28925</v>
       </c>
-      <c r="G54" s="1">
+      <c r="K54" s="1">
         <v>33755</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>19</v>
       </c>
@@ -1961,20 +2312,28 @@
       <c r="C55" s="1">
         <v>126042</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D55" s="10">
+        <v>44648</v>
+      </c>
+      <c r="E55" s="1">
+        <v>81394</v>
+      </c>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1">
         <v>19760</v>
       </c>
-      <c r="E55" s="1">
+      <c r="I55" s="1">
         <v>1408.090909090909</v>
       </c>
-      <c r="F55" s="1">
+      <c r="J55" s="1">
         <v>4271</v>
       </c>
-      <c r="G55" s="1">
+      <c r="K55" s="1">
         <v>15489</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>20</v>
       </c>
@@ -1984,20 +2343,28 @@
       <c r="C56" s="1">
         <v>904078</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="10">
+        <v>546107</v>
+      </c>
+      <c r="E56" s="1">
+        <v>357971</v>
+      </c>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1">
         <v>140040</v>
       </c>
-      <c r="E56" s="1">
+      <c r="I56" s="1">
         <v>8187</v>
       </c>
-      <c r="F56" s="1">
+      <c r="J56" s="1">
         <v>49983</v>
       </c>
-      <c r="G56" s="1">
+      <c r="K56" s="1">
         <v>90057</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>21</v>
       </c>
@@ -2007,20 +2374,28 @@
       <c r="C57" s="1">
         <v>282614</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D57" s="10">
+        <v>144063</v>
+      </c>
+      <c r="E57" s="1">
+        <v>138551</v>
+      </c>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1">
         <v>43717</v>
       </c>
-      <c r="E57" s="1">
+      <c r="I57" s="1">
         <v>2079</v>
       </c>
-      <c r="F57" s="1">
+      <c r="J57" s="1">
         <v>20848</v>
       </c>
-      <c r="G57" s="1">
+      <c r="K57" s="1">
         <v>22869</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>22</v>
       </c>
@@ -2030,20 +2405,28 @@
       <c r="C58" s="1">
         <v>768179</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="10">
+        <v>452506</v>
+      </c>
+      <c r="E58" s="1">
+        <v>315673</v>
+      </c>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1">
         <v>119831</v>
       </c>
-      <c r="E58" s="1">
+      <c r="I58" s="1">
         <v>4627.272727272727</v>
       </c>
-      <c r="F58" s="1">
+      <c r="J58" s="1">
         <v>68931</v>
       </c>
-      <c r="G58" s="1">
+      <c r="K58" s="1">
         <v>50900</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>23</v>
       </c>
@@ -2053,20 +2436,28 @@
       <c r="C59" s="1">
         <v>566568</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D59" s="10">
+        <v>347852</v>
+      </c>
+      <c r="E59" s="1">
+        <v>218716</v>
+      </c>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1">
         <v>107374</v>
       </c>
-      <c r="E59" s="1">
+      <c r="I59" s="1">
         <v>5222.272727272727</v>
       </c>
-      <c r="F59" s="1">
+      <c r="J59" s="1">
         <v>49929</v>
       </c>
-      <c r="G59" s="1">
+      <c r="K59" s="1">
         <v>57445</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>24</v>
       </c>
@@ -2076,20 +2467,28 @@
       <c r="C60" s="1">
         <v>867169</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="10">
+        <v>550118</v>
+      </c>
+      <c r="E60" s="1">
+        <v>317051</v>
+      </c>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1">
         <v>148228</v>
       </c>
-      <c r="E60" s="1">
+      <c r="I60" s="1">
         <v>5876.909090909091</v>
       </c>
-      <c r="F60" s="1">
+      <c r="J60" s="1">
         <v>83582</v>
       </c>
-      <c r="G60" s="1">
+      <c r="K60" s="1">
         <v>64646</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>25</v>
       </c>
@@ -2099,20 +2498,28 @@
       <c r="C61" s="1">
         <v>253468</v>
       </c>
-      <c r="D61" s="1">
+      <c r="D61" s="10">
+        <v>141892</v>
+      </c>
+      <c r="E61" s="1">
+        <v>111576</v>
+      </c>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1">
         <v>49078</v>
       </c>
-      <c r="E61" s="1">
+      <c r="I61" s="1">
         <v>2652.3636363636365</v>
       </c>
-      <c r="F61" s="1">
+      <c r="J61" s="1">
         <v>19902</v>
       </c>
-      <c r="G61" s="1">
+      <c r="K61" s="1">
         <v>29176</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>26</v>
       </c>
@@ -2122,20 +2529,28 @@
       <c r="C62" s="1">
         <v>444216</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="10">
+        <v>273016</v>
+      </c>
+      <c r="E62" s="1">
+        <v>171200</v>
+      </c>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1">
         <v>67967</v>
       </c>
-      <c r="E62" s="1">
+      <c r="I62" s="1">
         <v>2280.2727272727275</v>
       </c>
-      <c r="F62" s="1">
+      <c r="J62" s="1">
         <v>42884</v>
       </c>
-      <c r="G62" s="1">
+      <c r="K62" s="1">
         <v>25083</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>27</v>
       </c>
@@ -2145,20 +2560,28 @@
       <c r="C63" s="1">
         <v>234640</v>
       </c>
-      <c r="D63" s="1">
+      <c r="D63" s="10">
+        <v>124133</v>
+      </c>
+      <c r="E63" s="1">
+        <v>110507</v>
+      </c>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1">
         <v>38051</v>
       </c>
-      <c r="E63" s="1">
+      <c r="I63" s="1">
         <v>1828.090909090909</v>
       </c>
-      <c r="F63" s="1">
+      <c r="J63" s="1">
         <v>17942</v>
       </c>
-      <c r="G63" s="1">
+      <c r="K63" s="1">
         <v>20109</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>28</v>
       </c>
@@ -2168,20 +2591,28 @@
       <c r="C64" s="1">
         <v>359823</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="10">
+        <v>175359</v>
+      </c>
+      <c r="E64" s="1">
+        <v>184464</v>
+      </c>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1">
         <v>56266</v>
       </c>
-      <c r="E64" s="1">
+      <c r="I64" s="1">
         <v>3246.2727272727275</v>
       </c>
-      <c r="F64" s="1">
+      <c r="J64" s="1">
         <v>20557</v>
       </c>
-      <c r="G64" s="1">
+      <c r="K64" s="1">
         <v>35709</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>29</v>
       </c>
@@ -2191,20 +2622,28 @@
       <c r="C65" s="1">
         <v>662114</v>
       </c>
-      <c r="D65" s="1">
+      <c r="D65" s="10">
+        <v>371619</v>
+      </c>
+      <c r="E65" s="1">
+        <v>290495</v>
+      </c>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1">
         <v>114961</v>
       </c>
-      <c r="E65" s="1">
+      <c r="I65" s="1">
         <v>6272.909090909091</v>
       </c>
-      <c r="F65" s="1">
+      <c r="J65" s="1">
         <v>45959</v>
       </c>
-      <c r="G65" s="1">
+      <c r="K65" s="1">
         <v>69002</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>30</v>
       </c>
@@ -2214,20 +2653,28 @@
       <c r="C66" s="1">
         <v>660311</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="10">
+        <v>415044</v>
+      </c>
+      <c r="E66" s="1">
+        <v>245267</v>
+      </c>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1">
         <v>118507</v>
       </c>
-      <c r="E66" s="1">
+      <c r="I66" s="1">
         <v>7772.636363636364</v>
       </c>
-      <c r="F66" s="1">
+      <c r="J66" s="1">
         <v>33008</v>
       </c>
-      <c r="G66" s="1">
+      <c r="K66" s="1">
         <v>85499</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>31</v>
       </c>
@@ -2237,20 +2684,28 @@
       <c r="C67" s="1">
         <v>425275</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="10">
+        <v>296284</v>
+      </c>
+      <c r="E67" s="1">
+        <v>128991</v>
+      </c>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1">
         <v>70409</v>
       </c>
-      <c r="E67" s="1">
+      <c r="I67" s="1">
         <v>2507.5454545454545</v>
       </c>
-      <c r="F67" s="1">
+      <c r="J67" s="1">
         <v>42826</v>
       </c>
-      <c r="G67" s="1">
+      <c r="K67" s="1">
         <v>27583</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>32</v>
       </c>
@@ -2260,20 +2715,28 @@
       <c r="C68" s="1">
         <v>467936</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="10">
+        <v>242696</v>
+      </c>
+      <c r="E68" s="1">
+        <v>225240</v>
+      </c>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1">
         <v>73266</v>
       </c>
-      <c r="E68" s="1">
+      <c r="I68" s="1">
         <v>3897.181818181818</v>
       </c>
-      <c r="F68" s="1">
+      <c r="J68" s="1">
         <v>30397</v>
       </c>
-      <c r="G68" s="1">
+      <c r="K68" s="1">
         <v>42869</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>33</v>
       </c>
@@ -2283,16 +2746,24 @@
       <c r="C69" s="1">
         <v>743917</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="10">
+        <v>466589</v>
+      </c>
+      <c r="E69" s="1">
+        <v>277328</v>
+      </c>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1">
         <v>122082</v>
       </c>
-      <c r="E69" s="1">
+      <c r="I69" s="1">
         <v>7146.363636363636</v>
       </c>
-      <c r="F69" s="1">
+      <c r="J69" s="1">
         <v>43472</v>
       </c>
-      <c r="G69" s="1">
+      <c r="K69" s="1">
         <v>78610</v>
       </c>
     </row>

</xml_diff>